<commit_message>
SWE.2: Phase 1 safety priority core architecture
Layered + ports-adapters + priority-rule-plugin-chain architecture
(13 elements SWA-01..13, 9 internal interfaces SWI-01..09) satisfying
SAFETY-REQ-0001..0009. New priority tiers (fire/ISOFIX/auto-lock/
ignition-off/driver command, planned for later phases) can be added
as a single new PriorityRule implementation registered in
EvaluationCycleOrchestrator's ordered registry, with no changes to
the arbitrator, existing rules, or gating layer. Updates ENG-TRC-001's
Architecture column.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/engineering/Traceability/ENG-TRC-001_양방향 요구사항 추적 매트릭스.xlsx
+++ b/deliverables/engineering/Traceability/ENG-TRC-001_양방향 요구사항 추적 매트릭스.xlsx
@@ -283,7 +283,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TPLTRC001ChangeHistoryTable" displayName="TPLTRC001ChangeHistoryTable" ref="A9:F10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TPLTRC001ChangeHistoryTable" displayName="TPLTRC001ChangeHistoryTable" ref="A9:F11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Revision"/>
     <x:tableColumn id="2" name="변경일"/>
@@ -700,7 +700,9 @@
       <c r="B10" s="42" t="str">
         <v>SAFETY-REQ-0001</v>
       </c>
-      <c r="C10" s="42" t="str"/>
+      <c r="C10" s="42" t="str">
+        <v>SWA-07, SWA-06, SWA-02</v>
+      </c>
       <c r="D10" s="42" t="str"/>
       <c r="E10" s="42" t="str"/>
       <c r="F10" s="42" t="str"/>
@@ -715,7 +717,9 @@
       <c r="B11" s="42" t="str">
         <v>SAFETY-REQ-0002</v>
       </c>
-      <c r="C11" s="42" t="str"/>
+      <c r="C11" s="42" t="str">
+        <v>SWA-06, SWA-07</v>
+      </c>
       <c r="D11" s="42" t="str"/>
       <c r="E11" s="42" t="str"/>
       <c r="F11" s="42" t="str"/>
@@ -730,7 +734,9 @@
       <c r="B12" s="42" t="str">
         <v>SAFETY-REQ-0003</v>
       </c>
-      <c r="C12" s="42" t="str"/>
+      <c r="C12" s="42" t="str">
+        <v>SWA-08</v>
+      </c>
       <c r="D12" s="42" t="str"/>
       <c r="E12" s="42" t="str"/>
       <c r="F12" s="42" t="str"/>
@@ -745,7 +751,9 @@
       <c r="B13" s="42" t="str">
         <v>SAFETY-REQ-0004</v>
       </c>
-      <c r="C13" s="42" t="str"/>
+      <c r="C13" s="42" t="str">
+        <v>SWA-08</v>
+      </c>
       <c r="D13" s="42" t="str"/>
       <c r="E13" s="42" t="str"/>
       <c r="F13" s="42" t="str"/>
@@ -760,7 +768,9 @@
       <c r="B14" s="42" t="str">
         <v>SAFETY-REQ-0005</v>
       </c>
-      <c r="C14" s="42" t="str"/>
+      <c r="C14" s="42" t="str">
+        <v>SWA-08</v>
+      </c>
       <c r="D14" s="42" t="str"/>
       <c r="E14" s="42" t="str"/>
       <c r="F14" s="42" t="str"/>
@@ -775,7 +785,9 @@
       <c r="B15" s="42" t="str">
         <v>SAFETY-REQ-0006</v>
       </c>
-      <c r="C15" s="42" t="str"/>
+      <c r="C15" s="42" t="str">
+        <v>SWA-04, SWA-12</v>
+      </c>
       <c r="D15" s="42" t="str"/>
       <c r="E15" s="42" t="str"/>
       <c r="F15" s="42" t="str"/>
@@ -790,7 +802,9 @@
       <c r="B16" s="42" t="str">
         <v>SAFETY-REQ-0007</v>
       </c>
-      <c r="C16" s="42" t="str"/>
+      <c r="C16" s="42" t="str">
+        <v>SWA-03</v>
+      </c>
       <c r="D16" s="42" t="str"/>
       <c r="E16" s="42" t="str"/>
       <c r="F16" s="42" t="str"/>
@@ -805,7 +819,9 @@
       <c r="B17" s="42" t="str">
         <v>SAFETY-REQ-0008</v>
       </c>
-      <c r="C17" s="42" t="str"/>
+      <c r="C17" s="42" t="str">
+        <v>SWA-09, SWA-11, SWA-05</v>
+      </c>
       <c r="D17" s="42" t="str"/>
       <c r="E17" s="42" t="str"/>
       <c r="F17" s="42" t="str"/>
@@ -820,7 +836,9 @@
       <c r="B18" s="42" t="str">
         <v>SAFETY-REQ-0009</v>
       </c>
-      <c r="C18" s="42" t="str"/>
+      <c r="C18" s="42" t="str">
+        <v>SWA-12, SWA-05</v>
+      </c>
       <c r="D18" s="42" t="str"/>
       <c r="E18" s="42" t="str"/>
       <c r="F18" s="42" t="str"/>
@@ -1016,6 +1034,26 @@
         <v>미승인(Draft)</v>
       </c>
     </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="42" t="str">
+        <v>0.2</v>
+      </c>
+      <c r="B11" s="42" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="C11" s="42" t="str">
+        <v>hk.yoon@hyundai-autoever.com</v>
+      </c>
+      <c r="D11" s="42" t="str">
+        <v>Phase 1 SWE.2 아키텍처 설계(ENG-SWE2-001/002) 완료에 따른 Architecture 컬럼(C10:C18) 갱신</v>
+      </c>
+      <c r="E11" s="42" t="str">
+        <v>초안, 미검토(Draft)</v>
+      </c>
+      <c r="F11" s="42" t="str">
+        <v>미승인(Draft)</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells>
     <mergeCell ref="A1:F2"/>

</xml_diff>

<commit_message>
SWE.2: Phase 1 safety priority core architecture (#3)
Layered + ports-adapters + priority-rule-plugin-chain architecture
(13 elements SWA-01..13, 9 internal interfaces SWI-01..09) satisfying
SAFETY-REQ-0001..0009. New priority tiers (fire/ISOFIX/auto-lock/
ignition-off/driver command, planned for later phases) can be added
as a single new PriorityRule implementation registered in
EvaluationCycleOrchestrator's ordered registry, with no changes to
the arbitrator, existing rules, or gating layer. Updates ENG-TRC-001's
Architecture column.

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/engineering/Traceability/ENG-TRC-001_양방향 요구사항 추적 매트릭스.xlsx
+++ b/deliverables/engineering/Traceability/ENG-TRC-001_양방향 요구사항 추적 매트릭스.xlsx
@@ -283,7 +283,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TPLTRC001ChangeHistoryTable" displayName="TPLTRC001ChangeHistoryTable" ref="A9:F10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TPLTRC001ChangeHistoryTable" displayName="TPLTRC001ChangeHistoryTable" ref="A9:F11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Revision"/>
     <x:tableColumn id="2" name="변경일"/>
@@ -700,7 +700,9 @@
       <c r="B10" s="42" t="str">
         <v>SAFETY-REQ-0001</v>
       </c>
-      <c r="C10" s="42" t="str"/>
+      <c r="C10" s="42" t="str">
+        <v>SWA-07, SWA-06, SWA-02</v>
+      </c>
       <c r="D10" s="42" t="str"/>
       <c r="E10" s="42" t="str"/>
       <c r="F10" s="42" t="str"/>
@@ -715,7 +717,9 @@
       <c r="B11" s="42" t="str">
         <v>SAFETY-REQ-0002</v>
       </c>
-      <c r="C11" s="42" t="str"/>
+      <c r="C11" s="42" t="str">
+        <v>SWA-06, SWA-07</v>
+      </c>
       <c r="D11" s="42" t="str"/>
       <c r="E11" s="42" t="str"/>
       <c r="F11" s="42" t="str"/>
@@ -730,7 +734,9 @@
       <c r="B12" s="42" t="str">
         <v>SAFETY-REQ-0003</v>
       </c>
-      <c r="C12" s="42" t="str"/>
+      <c r="C12" s="42" t="str">
+        <v>SWA-08</v>
+      </c>
       <c r="D12" s="42" t="str"/>
       <c r="E12" s="42" t="str"/>
       <c r="F12" s="42" t="str"/>
@@ -745,7 +751,9 @@
       <c r="B13" s="42" t="str">
         <v>SAFETY-REQ-0004</v>
       </c>
-      <c r="C13" s="42" t="str"/>
+      <c r="C13" s="42" t="str">
+        <v>SWA-08</v>
+      </c>
       <c r="D13" s="42" t="str"/>
       <c r="E13" s="42" t="str"/>
       <c r="F13" s="42" t="str"/>
@@ -760,7 +768,9 @@
       <c r="B14" s="42" t="str">
         <v>SAFETY-REQ-0005</v>
       </c>
-      <c r="C14" s="42" t="str"/>
+      <c r="C14" s="42" t="str">
+        <v>SWA-08</v>
+      </c>
       <c r="D14" s="42" t="str"/>
       <c r="E14" s="42" t="str"/>
       <c r="F14" s="42" t="str"/>
@@ -775,7 +785,9 @@
       <c r="B15" s="42" t="str">
         <v>SAFETY-REQ-0006</v>
       </c>
-      <c r="C15" s="42" t="str"/>
+      <c r="C15" s="42" t="str">
+        <v>SWA-04, SWA-12</v>
+      </c>
       <c r="D15" s="42" t="str"/>
       <c r="E15" s="42" t="str"/>
       <c r="F15" s="42" t="str"/>
@@ -790,7 +802,9 @@
       <c r="B16" s="42" t="str">
         <v>SAFETY-REQ-0007</v>
       </c>
-      <c r="C16" s="42" t="str"/>
+      <c r="C16" s="42" t="str">
+        <v>SWA-03</v>
+      </c>
       <c r="D16" s="42" t="str"/>
       <c r="E16" s="42" t="str"/>
       <c r="F16" s="42" t="str"/>
@@ -805,7 +819,9 @@
       <c r="B17" s="42" t="str">
         <v>SAFETY-REQ-0008</v>
       </c>
-      <c r="C17" s="42" t="str"/>
+      <c r="C17" s="42" t="str">
+        <v>SWA-09, SWA-11, SWA-05</v>
+      </c>
       <c r="D17" s="42" t="str"/>
       <c r="E17" s="42" t="str"/>
       <c r="F17" s="42" t="str"/>
@@ -820,7 +836,9 @@
       <c r="B18" s="42" t="str">
         <v>SAFETY-REQ-0009</v>
       </c>
-      <c r="C18" s="42" t="str"/>
+      <c r="C18" s="42" t="str">
+        <v>SWA-12, SWA-05</v>
+      </c>
       <c r="D18" s="42" t="str"/>
       <c r="E18" s="42" t="str"/>
       <c r="F18" s="42" t="str"/>
@@ -1016,6 +1034,26 @@
         <v>미승인(Draft)</v>
       </c>
     </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="42" t="str">
+        <v>0.2</v>
+      </c>
+      <c r="B11" s="42" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="C11" s="42" t="str">
+        <v>hk.yoon@hyundai-autoever.com</v>
+      </c>
+      <c r="D11" s="42" t="str">
+        <v>Phase 1 SWE.2 아키텍처 설계(ENG-SWE2-001/002) 완료에 따른 Architecture 컬럼(C10:C18) 갱신</v>
+      </c>
+      <c r="E11" s="42" t="str">
+        <v>초안, 미검토(Draft)</v>
+      </c>
+      <c r="F11" s="42" t="str">
+        <v>미승인(Draft)</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells>
     <mergeCell ref="A1:F2"/>

</xml_diff>